<commit_message>
refactoring validation active directory
</commit_message>
<xml_diff>
--- a/public/assets/import-templates/import-employees-template.xlsx
+++ b/public/assets/import-templates/import-employees-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\M\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mjd\mujdn-frontend\public\assets\import-templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B76FEC7-7181-41A8-A1C6-46765C5B0D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFB7B8E-E57E-429B-BF85-602173B487D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import Errors" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Email</t>
   </si>
@@ -62,6 +62,9 @@
   </si>
   <si>
     <t>IsActive</t>
+  </si>
+  <si>
+    <t>ActiveDirectoryUsername</t>
   </si>
 </sst>
 </file>
@@ -413,26 +416,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:O1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" customWidth="1"/>
-    <col min="3" max="3" width="11.453125" customWidth="1"/>
-    <col min="4" max="4" width="11.08984375" customWidth="1"/>
-    <col min="5" max="5" width="11.26953125" customWidth="1"/>
-    <col min="6" max="6" width="14.08984375" customWidth="1"/>
-    <col min="7" max="7" width="10.81640625" customWidth="1"/>
-    <col min="8" max="8" width="8.26953125" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="9.7265625" customWidth="1"/>
-    <col min="11" max="11" width="15.7265625" customWidth="1"/>
-    <col min="12" max="12" width="20.54296875" customWidth="1"/>
-    <col min="13" max="13" width="26.81640625" customWidth="1"/>
-    <col min="14" max="14" width="7.81640625" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" customWidth="1"/>
+    <col min="12" max="12" width="20.5703125" customWidth="1"/>
+    <col min="13" max="13" width="26.85546875" customWidth="1"/>
+    <col min="14" max="14" width="7.85546875" customWidth="1"/>
+    <col min="15" max="15" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -474,6 +478,9 @@
       </c>
       <c r="N1" s="1" t="s">
         <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixing import excel validation
</commit_message>
<xml_diff>
--- a/public/assets/import-templates/import-employees-template.xlsx
+++ b/public/assets/import-templates/import-employees-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mjd\mujdn-frontend\public\assets\import-templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFB7B8E-E57E-429B-BF85-602173B487D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF0D5BF-F73F-4E8A-B4C9-9FA37B5D00EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -86,7 +86,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -96,6 +96,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD3D3D3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -111,9 +117,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -420,39 +431,38 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" customWidth="1"/>
-    <col min="8" max="8" width="8.28515625" customWidth="1"/>
+    <col min="2" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="9.7109375" customWidth="1"/>
     <col min="11" max="11" width="15.7109375" customWidth="1"/>
-    <col min="12" max="12" width="20.5703125" customWidth="1"/>
+    <col min="12" max="12" width="20.5703125" style="2" customWidth="1"/>
     <col min="13" max="13" width="26.85546875" customWidth="1"/>
     <col min="14" max="14" width="7.85546875" customWidth="1"/>
     <col min="15" max="15" width="27" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -461,16 +471,16 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="1" t="s">

</xml_diff>

<commit_message>
fixing import excel issue and user validation
</commit_message>
<xml_diff>
--- a/public/assets/import-templates/import-employees-template.xlsx
+++ b/public/assets/import-templates/import-employees-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mjd\mujdn-frontend\public\assets\import-templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A1F8DD7-F3ED-4112-A405-46308C046868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAF66EAF-1160-489D-A9BD-DD8224349DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -86,7 +86,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -104,6 +104,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -117,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -125,6 +131,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,13 +455,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
@@ -462,7 +470,7 @@
       <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -489,7 +497,7 @@
       <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="7" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>